<commit_message>
fix(06_experimento): anonimiza nombres reales de evaluadores en datos_crudos
</commit_message>
<xml_diff>
--- a/06_Experimento/datos_crudos/MundiPets_Datos_Crudos_06_Experimento.xlsx
+++ b/06_Experimento/datos_crudos/MundiPets_Datos_Crudos_06_Experimento.xlsx
@@ -478,7 +478,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Clasificación individual de cada uno de los 3 expertos sobre cada requisito (183 filas = 61 requisitos × 3 evaluadores). Sin consolidar ni promediar.</t>
+          <t>Clasificación individual de cada uno de los 3 expertos sobre cada requisito (183 filas = 61 requisitos × 3 evaluadores). Sin consolidar ni promediar. Evaluadores identificados por código (EXP-01/02/03), no por nombre.</t>
         </is>
       </c>
     </row>
@@ -515,7 +515,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>evaluacion_expertos.csv y salida_detector.csv del repositorio MundiPets-PFC-IngReq (corpus actualizado a 61 requisitos, sincronizado con instrumentos/rubrica_clasificacion_experta.xlsx).</t>
+          <t>evaluacion_expertos.csv y salida_detector.csv del repositorio MundiPets-PFC-IngReq (corpus de 61 requisitos, evaluadores anonimizados por código).</t>
         </is>
       </c>
     </row>
@@ -541,7 +541,7 @@
     <col width="28" customWidth="1" min="6" max="6"/>
     <col width="45" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="32" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
@@ -640,7 +640,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -692,7 +692,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -744,7 +744,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -796,7 +796,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -848,7 +848,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -900,7 +900,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -952,7 +952,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -1004,7 +1004,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -1056,7 +1056,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -1108,7 +1108,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1160,7 +1160,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1212,7 +1212,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1264,7 +1264,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1316,7 +1316,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1368,7 +1368,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1420,7 +1420,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -1472,7 +1472,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -1524,7 +1524,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -1576,7 +1576,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -1628,7 +1628,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -1680,7 +1680,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -1732,7 +1732,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -1784,7 +1784,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -1836,7 +1836,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -1888,7 +1888,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -1940,7 +1940,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -1992,7 +1992,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -2044,7 +2044,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -2148,7 +2148,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -2200,7 +2200,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -2252,7 +2252,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -2304,7 +2304,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
@@ -2356,7 +2356,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -2408,7 +2408,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -2460,7 +2460,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -2512,7 +2512,7 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
@@ -2564,7 +2564,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -2616,7 +2616,7 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
@@ -2668,7 +2668,7 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
@@ -2720,7 +2720,7 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
@@ -2772,7 +2772,7 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -2824,7 +2824,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
@@ -2876,7 +2876,7 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -2928,7 +2928,7 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
@@ -2980,7 +2980,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
@@ -3032,7 +3032,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -3084,7 +3084,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
@@ -3136,7 +3136,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -3188,7 +3188,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -3240,7 +3240,7 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -3292,7 +3292,7 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -3344,7 +3344,7 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -3396,7 +3396,7 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -3448,7 +3448,7 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
@@ -3500,7 +3500,7 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
@@ -3552,7 +3552,7 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
@@ -3604,7 +3604,7 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
@@ -3656,7 +3656,7 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
@@ -3708,7 +3708,7 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
@@ -3760,7 +3760,7 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>Angélica Michelle Tenecela Intriago</t>
+          <t>EXP-01</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
@@ -3812,7 +3812,7 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
@@ -3864,7 +3864,7 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
@@ -3916,7 +3916,7 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
@@ -3968,7 +3968,7 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
@@ -4020,7 +4020,7 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
@@ -4072,7 +4072,7 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
@@ -4124,7 +4124,7 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
@@ -4176,7 +4176,7 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
@@ -4228,7 +4228,7 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
@@ -4280,7 +4280,7 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
@@ -4332,7 +4332,7 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
@@ -4384,7 +4384,7 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
@@ -4436,7 +4436,7 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
@@ -4488,7 +4488,7 @@
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
@@ -4540,7 +4540,7 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
@@ -4592,7 +4592,7 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
@@ -4644,7 +4644,7 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
@@ -4696,7 +4696,7 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
@@ -4748,7 +4748,7 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
@@ -4800,7 +4800,7 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
@@ -4852,7 +4852,7 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
@@ -4904,7 +4904,7 @@
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J84" t="inlineStr">
@@ -4956,7 +4956,7 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
@@ -5008,7 +5008,7 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J86" t="inlineStr">
@@ -5060,7 +5060,7 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
@@ -5112,7 +5112,7 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
@@ -5164,7 +5164,7 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
@@ -5216,7 +5216,7 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J90" t="inlineStr">
@@ -5268,7 +5268,7 @@
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
@@ -5320,7 +5320,7 @@
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J92" t="inlineStr">
@@ -5372,7 +5372,7 @@
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
@@ -5424,7 +5424,7 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J94" t="inlineStr">
@@ -5476,7 +5476,7 @@
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
@@ -5528,7 +5528,7 @@
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J96" t="inlineStr">
@@ -5580,7 +5580,7 @@
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
@@ -5632,7 +5632,7 @@
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J98" t="inlineStr">
@@ -5684,7 +5684,7 @@
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
@@ -5736,7 +5736,7 @@
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J100" t="inlineStr">
@@ -5788,7 +5788,7 @@
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
@@ -5840,7 +5840,7 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J102" t="inlineStr">
@@ -5892,7 +5892,7 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
@@ -5944,7 +5944,7 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
@@ -5996,7 +5996,7 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
@@ -6048,7 +6048,7 @@
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J106" t="inlineStr">
@@ -6100,7 +6100,7 @@
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J107" t="inlineStr">
@@ -6152,7 +6152,7 @@
       </c>
       <c r="I108" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J108" t="inlineStr">
@@ -6204,7 +6204,7 @@
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J109" t="inlineStr">
@@ -6256,7 +6256,7 @@
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J110" t="inlineStr">
@@ -6308,7 +6308,7 @@
       </c>
       <c r="I111" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
@@ -6360,7 +6360,7 @@
       </c>
       <c r="I112" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
@@ -6412,7 +6412,7 @@
       </c>
       <c r="I113" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J113" t="inlineStr">
@@ -6464,7 +6464,7 @@
       </c>
       <c r="I114" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J114" t="inlineStr">
@@ -6516,7 +6516,7 @@
       </c>
       <c r="I115" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J115" t="inlineStr">
@@ -6568,7 +6568,7 @@
       </c>
       <c r="I116" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J116" t="inlineStr">
@@ -6620,7 +6620,7 @@
       </c>
       <c r="I117" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J117" t="inlineStr">
@@ -6672,7 +6672,7 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J118" t="inlineStr">
@@ -6724,7 +6724,7 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J119" t="inlineStr">
@@ -6776,7 +6776,7 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
@@ -6828,7 +6828,7 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
@@ -6880,7 +6880,7 @@
       </c>
       <c r="I122" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J122" t="inlineStr">
@@ -6932,7 +6932,7 @@
       </c>
       <c r="I123" t="inlineStr">
         <is>
-          <t>Geovanny Alexander Ochoa Gilces</t>
+          <t>EXP-02</t>
         </is>
       </c>
       <c r="J123" t="inlineStr">
@@ -6984,7 +6984,7 @@
       </c>
       <c r="I124" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J124" t="inlineStr">
@@ -7036,7 +7036,7 @@
       </c>
       <c r="I125" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
@@ -7088,7 +7088,7 @@
       </c>
       <c r="I126" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J126" t="inlineStr">
@@ -7140,7 +7140,7 @@
       </c>
       <c r="I127" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J127" t="inlineStr">
@@ -7192,7 +7192,7 @@
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J128" t="inlineStr">
@@ -7244,7 +7244,7 @@
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
@@ -7296,7 +7296,7 @@
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J130" t="inlineStr">
@@ -7348,7 +7348,7 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
@@ -7400,7 +7400,7 @@
       </c>
       <c r="I132" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J132" t="inlineStr">
@@ -7452,7 +7452,7 @@
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J133" t="inlineStr">
@@ -7504,7 +7504,7 @@
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J134" t="inlineStr">
@@ -7556,7 +7556,7 @@
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J135" t="inlineStr">
@@ -7608,7 +7608,7 @@
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J136" t="inlineStr">
@@ -7660,7 +7660,7 @@
       </c>
       <c r="I137" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J137" t="inlineStr">
@@ -7712,7 +7712,7 @@
       </c>
       <c r="I138" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J138" t="inlineStr">
@@ -7764,7 +7764,7 @@
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J139" t="inlineStr">
@@ -7816,7 +7816,7 @@
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J140" t="inlineStr">
@@ -7868,7 +7868,7 @@
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J141" t="inlineStr">
@@ -7920,7 +7920,7 @@
       </c>
       <c r="I142" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J142" t="inlineStr">
@@ -7972,7 +7972,7 @@
       </c>
       <c r="I143" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J143" t="inlineStr">
@@ -8024,7 +8024,7 @@
       </c>
       <c r="I144" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J144" t="inlineStr">
@@ -8076,7 +8076,7 @@
       </c>
       <c r="I145" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J145" t="inlineStr">
@@ -8128,7 +8128,7 @@
       </c>
       <c r="I146" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J146" t="inlineStr">
@@ -8180,7 +8180,7 @@
       </c>
       <c r="I147" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J147" t="inlineStr">
@@ -8232,7 +8232,7 @@
       </c>
       <c r="I148" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J148" t="inlineStr">
@@ -8284,7 +8284,7 @@
       </c>
       <c r="I149" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J149" t="inlineStr">
@@ -8336,7 +8336,7 @@
       </c>
       <c r="I150" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J150" t="inlineStr">
@@ -8388,7 +8388,7 @@
       </c>
       <c r="I151" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J151" t="inlineStr">
@@ -8440,7 +8440,7 @@
       </c>
       <c r="I152" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J152" t="inlineStr">
@@ -8492,7 +8492,7 @@
       </c>
       <c r="I153" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J153" t="inlineStr">
@@ -8544,7 +8544,7 @@
       </c>
       <c r="I154" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J154" t="inlineStr">
@@ -8596,7 +8596,7 @@
       </c>
       <c r="I155" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J155" t="inlineStr">
@@ -8648,7 +8648,7 @@
       </c>
       <c r="I156" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J156" t="inlineStr">
@@ -8700,7 +8700,7 @@
       </c>
       <c r="I157" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J157" t="inlineStr">
@@ -8752,7 +8752,7 @@
       </c>
       <c r="I158" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J158" t="inlineStr">
@@ -8804,7 +8804,7 @@
       </c>
       <c r="I159" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J159" t="inlineStr">
@@ -8856,7 +8856,7 @@
       </c>
       <c r="I160" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J160" t="inlineStr">
@@ -8908,7 +8908,7 @@
       </c>
       <c r="I161" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J161" t="inlineStr">
@@ -8960,7 +8960,7 @@
       </c>
       <c r="I162" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J162" t="inlineStr">
@@ -9012,7 +9012,7 @@
       </c>
       <c r="I163" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J163" t="inlineStr">
@@ -9064,7 +9064,7 @@
       </c>
       <c r="I164" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J164" t="inlineStr">
@@ -9116,7 +9116,7 @@
       </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J165" t="inlineStr">
@@ -9168,7 +9168,7 @@
       </c>
       <c r="I166" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J166" t="inlineStr">
@@ -9220,7 +9220,7 @@
       </c>
       <c r="I167" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J167" t="inlineStr">
@@ -9272,7 +9272,7 @@
       </c>
       <c r="I168" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J168" t="inlineStr">
@@ -9324,7 +9324,7 @@
       </c>
       <c r="I169" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J169" t="inlineStr">
@@ -9376,7 +9376,7 @@
       </c>
       <c r="I170" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J170" t="inlineStr">
@@ -9428,7 +9428,7 @@
       </c>
       <c r="I171" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J171" t="inlineStr">
@@ -9480,7 +9480,7 @@
       </c>
       <c r="I172" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J172" t="inlineStr">
@@ -9532,7 +9532,7 @@
       </c>
       <c r="I173" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J173" t="inlineStr">
@@ -9584,7 +9584,7 @@
       </c>
       <c r="I174" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J174" t="inlineStr">
@@ -9636,7 +9636,7 @@
       </c>
       <c r="I175" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J175" t="inlineStr">
@@ -9688,7 +9688,7 @@
       </c>
       <c r="I176" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J176" t="inlineStr">
@@ -9740,7 +9740,7 @@
       </c>
       <c r="I177" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J177" t="inlineStr">
@@ -9792,7 +9792,7 @@
       </c>
       <c r="I178" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J178" t="inlineStr">
@@ -9844,7 +9844,7 @@
       </c>
       <c r="I179" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J179" t="inlineStr">
@@ -9896,7 +9896,7 @@
       </c>
       <c r="I180" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J180" t="inlineStr">
@@ -9948,7 +9948,7 @@
       </c>
       <c r="I181" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J181" t="inlineStr">
@@ -10000,7 +10000,7 @@
       </c>
       <c r="I182" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J182" t="inlineStr">
@@ -10052,7 +10052,7 @@
       </c>
       <c r="I183" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J183" t="inlineStr">
@@ -10104,7 +10104,7 @@
       </c>
       <c r="I184" t="inlineStr">
         <is>
-          <t>Valeska Sofía Chica Valfré</t>
+          <t>EXP-03</t>
         </is>
       </c>
       <c r="J184" t="inlineStr">

</xml_diff>